<commit_message>
pénzes excel - Marci
</commit_message>
<xml_diff>
--- a/pénzes_excel.xlsx
+++ b/pénzes_excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BME\MSC_SEM_2\RobonAutism\Robonaut\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e5ee7a4626f47f2/MSc/2. félév_M/RobonAut/RobonAut/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187ACD52-3E74-47C5-BD30-30EA4FB25B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{187ACD52-3E74-47C5-BD30-30EA4FB25B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D521CF57-FB58-47F8-A959-A4FA7E60D655}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1695" windowWidth="21600" windowHeight="11085" xr2:uid="{EF0642E4-593F-4BBF-8839-D4AD9E30F0ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EF0642E4-593F-4BBF-8839-D4AD9E30F0ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Dávid</t>
   </si>
@@ -60,6 +60,15 @@
   </si>
   <si>
     <t>Motormeghajtó kártya</t>
+  </si>
+  <si>
+    <t>Breadboard</t>
+  </si>
+  <si>
+    <t>Jumper Kábel</t>
+  </si>
+  <si>
+    <t>lipo save</t>
   </si>
 </sst>
 </file>
@@ -102,9 +111,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -120,6 +132,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -439,14 +455,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7560C3A4-8E38-490B-8570-812DE0470CF7}">
-  <dimension ref="A2:E5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A2:E8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.19921875" customWidth="1"/>
-    <col min="5" max="5" width="12.06640625" customWidth="1"/>
+    <col min="1" max="1" width="18.21875" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -463,7 +479,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -471,7 +487,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -479,7 +495,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -487,7 +503,32 @@
         <v>12000</v>
       </c>
     </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2535</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <v>5390</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C6:C7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>